<commit_message>
2.0 Wrap-Up (part 2) - Did a full review of the semantics of all YAML options, making a large number of adjustments (some small, some larger). 2 of the more notable changes were: 	- Adjusted double_gems to work when just shop_randomization is on, not only when gem_logic is on. 	- Renamed "off" to "vanilla" for open_world_mode. - Fixed gem amounts slightly - mismarked the steel traps in Gloomy Glacier as not being enemies when they are.
</commit_message>
<xml_diff>
--- a/worlds/spyro_aht/setup/Gem Research.xlsx
+++ b/worlds/spyro_aht/setup/Gem Research.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sean\Downloads\Archipelago Stuff\.apworlds\PhoenixAP\worlds\spyro_aht\setup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sean\Downloads\Archipelago Stuff\apworlds\PhoenixAP\worlds\spyro_aht\setup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231CD9C6-0017-4852-8B2E-17C12C05CF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A528B702-1771-4E26-A2C5-616CCEBB35D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="697" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="697" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="New Gems (simplified per-rule)" sheetId="14" r:id="rId1"/>
@@ -2174,9 +2174,6 @@
     <t>frozen gem blocks via exploding arrows</t>
   </si>
   <si>
-    <t>steel traps via exploding arrows</t>
-  </si>
-  <si>
     <t>armored chests</t>
   </si>
   <si>
@@ -2436,6 +2433,9 @@
   </si>
   <si>
     <t>OTHER</t>
+  </si>
+  <si>
+    <t>[enemy] steel traps via exploding arrows</t>
   </si>
 </sst>
 </file>
@@ -13950,7 +13950,7 @@
     </row>
     <row r="804" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A804" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B804" s="1">
         <v>16153</v>
@@ -13958,7 +13958,7 @@
     </row>
     <row r="805" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A805" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B805" s="1">
         <f>B802-B803-B804</f>
@@ -14082,7 +14082,7 @@
         <v>396</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>21</v>
@@ -14138,7 +14138,7 @@
         <v>335</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>21</v>
@@ -14167,7 +14167,7 @@
         <v>215</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>21</v>
@@ -14182,7 +14182,7 @@
         <v>286</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>21</v>
@@ -14225,7 +14225,7 @@
         <v>451</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>21</v>
@@ -14399,7 +14399,7 @@
         <v>260</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>50</v>
@@ -14498,7 +14498,7 @@
         <v>205</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>21</v>
@@ -14582,7 +14582,7 @@
         <v>175</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>21</v>
@@ -14835,7 +14835,7 @@
         <v>105</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>21</v>
@@ -15122,7 +15122,7 @@
         <v>223</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>21</v>
@@ -15234,7 +15234,7 @@
         <v>330</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>21</v>
@@ -15305,7 +15305,7 @@
         <v>994</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>21</v>
@@ -15319,7 +15319,7 @@
         <v>275</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>21</v>
@@ -15717,7 +15717,7 @@
         <v>175</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D126" s="1" t="s">
         <v>36</v>
@@ -15773,7 +15773,7 @@
         <v>40</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D130" s="1" t="s">
         <v>50</v>
@@ -15788,7 +15788,7 @@
         <v>303</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D131" s="1" t="s">
         <v>21</v>
@@ -15858,7 +15858,7 @@
         <v>2020</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D136" s="1" t="s">
         <v>68</v>
@@ -15872,7 +15872,7 @@
         <v>1050</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D137" s="1" t="s">
         <v>226</v>
@@ -15915,7 +15915,7 @@
         <v>525</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D140" s="1" t="s">
         <v>21</v>
@@ -15985,7 +15985,7 @@
         <v>388</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="D145" s="1" t="s">
         <v>228</v>
@@ -16056,7 +16056,7 @@
         <v>115</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="D150" s="1" t="s">
         <v>50</v>
@@ -16154,7 +16154,7 @@
         <v>120</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="D157" s="1" t="s">
         <v>50</v>
@@ -16371,7 +16371,7 @@
         <v>180</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="D173" s="1" t="s">
         <v>21</v>
@@ -16554,7 +16554,7 @@
         <v>755</v>
       </c>
       <c r="C186" s="1" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D186" s="1" t="s">
         <v>21</v>
@@ -16610,7 +16610,7 @@
         <v>85</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D190" s="1" t="s">
         <v>21</v>
@@ -16639,7 +16639,7 @@
         <v>280</v>
       </c>
       <c r="C192" s="1" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D192" s="1" t="s">
         <v>21</v>
@@ -16682,7 +16682,7 @@
         <v>225</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D195" s="1" t="s">
         <v>234</v>
@@ -16842,7 +16842,7 @@
         <v>125</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D207" s="1" t="s">
         <v>50</v>
@@ -16955,7 +16955,7 @@
         <v>397</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D215" s="1" t="s">
         <v>68</v>
@@ -17377,7 +17377,7 @@
         <v>246</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D245" s="1" t="s">
         <v>21</v>
@@ -17406,7 +17406,7 @@
         <v>205</v>
       </c>
       <c r="C247" s="1" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D247" s="1" t="s">
         <v>21</v>
@@ -17435,7 +17435,7 @@
         <v>513</v>
       </c>
       <c r="C249" s="1" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D249" s="1" t="s">
         <v>21</v>
@@ -17576,7 +17576,7 @@
         <v>250</v>
       </c>
       <c r="C259" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D259" s="1" t="s">
         <v>21</v>
@@ -17591,7 +17591,7 @@
         <v>342</v>
       </c>
       <c r="C260" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D260" s="1" t="s">
         <v>21</v>
@@ -17638,7 +17638,7 @@
         <v>100</v>
       </c>
       <c r="C264" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D264" s="1" t="s">
         <v>21</v>
@@ -17736,7 +17736,7 @@
         <v>145</v>
       </c>
       <c r="C271" s="1" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D271" s="1" t="s">
         <v>50</v>
@@ -17765,7 +17765,7 @@
         <v>1016</v>
       </c>
       <c r="C273" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D273" s="1" t="s">
         <v>21</v>
@@ -17891,7 +17891,7 @@
         <v>141</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D282" s="1" t="s">
         <v>23</v>
@@ -17905,7 +17905,7 @@
         <v>571</v>
       </c>
       <c r="C283" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D283" s="1" t="s">
         <v>21</v>
@@ -18061,7 +18061,7 @@
         <v>1166</v>
       </c>
       <c r="C294" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D294" s="1" t="s">
         <v>21</v>
@@ -18299,7 +18299,7 @@
         <v>160</v>
       </c>
       <c r="C311" s="1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D311" s="1" t="s">
         <v>307</v>
@@ -18346,7 +18346,7 @@
         <v>656</v>
       </c>
       <c r="C315" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D315" s="1" t="s">
         <v>21</v>
@@ -18402,7 +18402,7 @@
         <v>200</v>
       </c>
       <c r="C319" s="1" t="s">
-        <v>569</v>
+        <v>656</v>
       </c>
       <c r="D319" s="1" t="s">
         <v>21</v>
@@ -18603,7 +18603,7 @@
         <v>40</v>
       </c>
       <c r="C334" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D334" s="1" t="s">
         <v>50</v>
@@ -18617,7 +18617,7 @@
         <v>175</v>
       </c>
       <c r="C335" s="1" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D335" s="1" t="s">
         <v>21</v>
@@ -18659,7 +18659,7 @@
         <v>39</v>
       </c>
       <c r="C338" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D338" s="1" t="s">
         <v>50</v>
@@ -18674,7 +18674,7 @@
         <v>475</v>
       </c>
       <c r="C339" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D339" s="1" t="s">
         <v>21</v>
@@ -18731,7 +18731,7 @@
         <v>208</v>
       </c>
       <c r="C343" s="1" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D343" s="1" t="s">
         <v>21</v>
@@ -18871,7 +18871,7 @@
         <v>140</v>
       </c>
       <c r="C353" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D353" s="1" t="s">
         <v>50</v>
@@ -18899,7 +18899,7 @@
         <v>1500</v>
       </c>
       <c r="C355" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D355" s="1" t="s">
         <v>21</v>
@@ -18913,7 +18913,7 @@
         <v>325</v>
       </c>
       <c r="C356" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D356" s="1" t="s">
         <v>21</v>
@@ -19081,7 +19081,7 @@
         <v>60</v>
       </c>
       <c r="C368" s="1" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D368" s="1" t="s">
         <v>21</v>
@@ -19109,7 +19109,7 @@
         <v>5000</v>
       </c>
       <c r="C370" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D370" s="1" t="s">
         <v>21</v>
@@ -19165,7 +19165,7 @@
         <v>150</v>
       </c>
       <c r="C374" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D374" s="1" t="s">
         <v>21</v>
@@ -19180,7 +19180,7 @@
         <v>296</v>
       </c>
       <c r="C375" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D375" s="1" t="s">
         <v>21</v>
@@ -19194,7 +19194,7 @@
         <v>80</v>
       </c>
       <c r="C376" s="1" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D376" s="1" t="s">
         <v>23</v>
@@ -19396,7 +19396,7 @@
         <v>1414</v>
       </c>
       <c r="C391" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D391" s="1" t="s">
         <v>21</v>
@@ -19438,7 +19438,7 @@
         <v>40</v>
       </c>
       <c r="C394" s="1" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D394" s="1" t="s">
         <v>50</v>
@@ -19541,7 +19541,7 @@
         <v>572</v>
       </c>
       <c r="C402" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D402" s="1" t="s">
         <v>21</v>
@@ -19555,7 +19555,7 @@
         <v>161</v>
       </c>
       <c r="C403" s="1" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D403" s="1" t="s">
         <v>21</v>
@@ -19569,7 +19569,7 @@
         <v>100</v>
       </c>
       <c r="C404" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D404" s="1" t="s">
         <v>400</v>
@@ -19822,7 +19822,7 @@
         <v>235</v>
       </c>
       <c r="C422" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D422" s="1" t="s">
         <v>21</v>
@@ -19934,7 +19934,7 @@
         <v>160</v>
       </c>
       <c r="C430" s="1" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D430" s="1" t="s">
         <v>21</v>
@@ -19949,7 +19949,7 @@
         <v>300</v>
       </c>
       <c r="C431" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D431" s="1" t="s">
         <v>400</v>
@@ -20020,7 +20020,7 @@
         <v>154</v>
       </c>
       <c r="C436" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D436" s="1" t="s">
         <v>21</v>
@@ -20048,7 +20048,7 @@
         <v>75</v>
       </c>
       <c r="C438" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D438" s="1" t="s">
         <v>21</v>
@@ -20063,7 +20063,7 @@
         <v>750</v>
       </c>
       <c r="C439" s="1" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D439" s="1" t="s">
         <v>21</v>
@@ -20148,7 +20148,7 @@
         <v>658</v>
       </c>
       <c r="C445" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D445" s="1" t="s">
         <v>21</v>
@@ -20191,7 +20191,7 @@
         <v>890</v>
       </c>
       <c r="C448" s="1" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D448" s="1" t="s">
         <v>23</v>
@@ -20220,7 +20220,7 @@
         <v>373</v>
       </c>
       <c r="C450" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D450" s="1" t="s">
         <v>21</v>
@@ -20450,7 +20450,7 @@
         <v>125</v>
       </c>
       <c r="C467" s="1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D467" s="1" t="s">
         <v>21</v>
@@ -20464,7 +20464,7 @@
         <v>500</v>
       </c>
       <c r="C468" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D468" s="1" t="s">
         <v>40</v>
@@ -20931,7 +20931,7 @@
         <v>150</v>
       </c>
       <c r="C502" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D502" s="1" t="s">
         <v>408</v>
@@ -20959,7 +20959,7 @@
         <v>100</v>
       </c>
       <c r="C504" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D504" s="1" t="s">
         <v>23</v>
@@ -21001,7 +21001,7 @@
         <v>110</v>
       </c>
       <c r="C507" s="1" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D507" s="1" t="s">
         <v>408</v>
@@ -21072,7 +21072,7 @@
         <v>530</v>
       </c>
       <c r="C512" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D512" s="1" t="s">
         <v>21</v>
@@ -21171,7 +21171,7 @@
         <v>285</v>
       </c>
       <c r="C519" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D519" s="1" t="s">
         <v>21</v>
@@ -21186,7 +21186,7 @@
         <v>540</v>
       </c>
       <c r="C520" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D520" s="1" t="s">
         <v>21</v>
@@ -21228,7 +21228,7 @@
         <v>195</v>
       </c>
       <c r="C523" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D523" s="1" t="s">
         <v>408</v>
@@ -21242,7 +21242,7 @@
         <v>105</v>
       </c>
       <c r="C524" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D524" s="1" t="s">
         <v>21</v>
@@ -21270,7 +21270,7 @@
         <v>60</v>
       </c>
       <c r="C526" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D526" s="1" t="s">
         <v>415</v>
@@ -21285,7 +21285,7 @@
         <v>185</v>
       </c>
       <c r="C527" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D527" s="1" t="s">
         <v>408</v>
@@ -21327,7 +21327,7 @@
         <v>275</v>
       </c>
       <c r="C530" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D530" s="1" t="s">
         <v>21</v>
@@ -21355,7 +21355,7 @@
         <v>160</v>
       </c>
       <c r="C532" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D532" s="1" t="s">
         <v>21</v>
@@ -21389,7 +21389,7 @@
         <v>868</v>
       </c>
       <c r="C535" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D535" s="1" t="s">
         <v>21</v>
@@ -21403,7 +21403,7 @@
         <v>80</v>
       </c>
       <c r="C536" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D536" s="1" t="s">
         <v>21</v>
@@ -21431,7 +21431,7 @@
         <v>55</v>
       </c>
       <c r="C538" s="1" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D538" s="1" t="s">
         <v>23</v>
@@ -21459,7 +21459,7 @@
         <v>60</v>
       </c>
       <c r="C540" s="1" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D540" s="1" t="s">
         <v>36</v>
@@ -21487,7 +21487,7 @@
         <v>60</v>
       </c>
       <c r="C542" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D542" s="1" t="s">
         <v>408</v>
@@ -21543,7 +21543,7 @@
         <v>60</v>
       </c>
       <c r="C546" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D546" s="1" t="s">
         <v>21</v>
@@ -21656,7 +21656,7 @@
         <v>155</v>
       </c>
       <c r="C554" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D554" s="1" t="s">
         <v>21</v>
@@ -21712,7 +21712,7 @@
         <v>80</v>
       </c>
       <c r="C558" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D558" s="1" t="s">
         <v>21</v>
@@ -21811,7 +21811,7 @@
         <v>345</v>
       </c>
       <c r="C565" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D565" s="1" t="s">
         <v>36</v>
@@ -21895,7 +21895,7 @@
         <v>105</v>
       </c>
       <c r="C571" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D571" s="1" t="s">
         <v>36</v>
@@ -22078,7 +22078,7 @@
     </row>
     <row r="586" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A586" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B586" s="1">
         <v>16153</v>
@@ -22086,7 +22086,7 @@
     </row>
     <row r="587" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A587" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B587" s="1">
         <f>B584-B585-B586</f>

</xml_diff>